<commit_message>
test(v7): verify new artwork and refresh backend handoff
</commit_message>
<xml_diff>
--- a/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
+++ b/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="Rcf01fd260f834a32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="R0ceed03d7cb94064"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="Rd458340b4fd44f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="Rd851d07fb3bb42fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="R2e3522c4bf7c41ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R7025cc702ba3414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="R1e450220f29c480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="Re3654206f651406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="R9cae78a492644e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="R032d57a7fee34c44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="R003c50fd1d8547c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R509fae8fdbe84437"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -609,7 +609,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -695,16 +695,16 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
-        <x:v>["v7-1","v7-2"]</x:v>
+        <x:v>["v7-1","v7-2","v7-3"]</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str">
         <x:v>作品 DesignConfig</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>默认v7-2；旧作品v7-1按原版本回放</x:v>
+        <x:v>默认v7-3；旧作品v7-1/v7-2按原版本回放</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="55" customHeight="1">
@@ -1180,7 +1180,7 @@
         <x:v>深圳默认作品 JSON（H列完整复制）</x:v>
       </x:c>
       <x:c r="H28" s="12" t="str">
-        <x:v>{"schemaVersion":1,"resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","cityId":"shenzhen","sloganId":"open","appearance":{"preset":"gold","hue":41.80851063829786,"saturation":100,"lightness":63.13725490196078,"material":1,"materialX":0.5,"relief":1}}</x:v>
+        <x:v>{"schemaVersion":1,"resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","cityId":"shenzhen","sloganId":"open","appearance":{"preset":"gold","hue":41.80851063829786,"saturation":100,"lightness":63.13725490196078,"material":1,"materialX":0.5,"relief":1}}</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="34" customHeight="1">
@@ -1188,73 +1188,88 @@
         <x:v>数据来源（完整提交与文件哈希见JSON sources）</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/package.json</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
       <x:c r="H31" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/styles/slogans.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/evidence/v7.1.2/slogans-source.json</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
       <x:c r="H32" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/evidence/v7.1.2/cities/review.json</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
       <x:c r="H33" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
       <x:c r="H34" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/slogans.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
       <x:c r="H35" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
       <x:c r="H36" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/resources/types.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="H37" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/resources/design.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="H38" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="H39" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/types.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="H40" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/design.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
       <x:c r="H41" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/public/releases/v7-2/catalog.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="H42" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/ec6f9bb0b606f319435f57dc18fbc6375ed6566a/guangcai-china-preview/public/releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="H43" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="H44" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/releases/v7-3/catalog.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="H45" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2f456ad1a174b07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R784db46361f04a5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1312,7 +1327,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1394,10 +1409,10 @@
         <x:v>上海</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>shanghai-thumbnail</x:v>
@@ -1421,7 +1436,7 @@
         <x:v>shanghai-detail-normal</x:v>
       </x:c>
       <x:c r="M6" s="10" t="str">
-        <x:v>{"cityId":"shanghai","name":"上海","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"shanghai-thumbnail","light":{"mask":"shanghai-light-mask","normal":"shanghai-light-normal"},"standard":{"mask":"shanghai-standard-mask","normal":"shanghai-standard-normal"},"detail":{"mask":"shanghai-detail-mask","normal":"shanghai-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shanghai","name":"上海","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shanghai-thumbnail","light":{"mask":"shanghai-light-mask","normal":"shanghai-light-normal"},"standard":{"mask":"shanghai-standard-mask","normal":"shanghai-standard-normal"},"detail":{"mask":"shanghai-detail-mask","normal":"shanghai-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
@@ -1435,10 +1450,10 @@
         <x:v>乌鲁木齐</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
         <x:v>urumqi-thumbnail</x:v>
@@ -1462,7 +1477,7 @@
         <x:v>urumqi-detail-normal</x:v>
       </x:c>
       <x:c r="M7" s="11" t="str">
-        <x:v>{"cityId":"urumqi","name":"乌鲁木齐","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"urumqi-thumbnail","light":{"mask":"urumqi-light-mask","normal":"urumqi-light-normal"},"standard":{"mask":"urumqi-standard-mask","normal":"urumqi-standard-normal"},"detail":{"mask":"urumqi-detail-mask","normal":"urumqi-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"urumqi","name":"乌鲁木齐","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"urumqi-thumbnail","light":{"mask":"urumqi-light-mask","normal":"urumqi-light-normal"},"standard":{"mask":"urumqi-standard-mask","normal":"urumqi-standard-normal"},"detail":{"mask":"urumqi-detail-mask","normal":"urumqi-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
@@ -1476,10 +1491,10 @@
         <x:v>北京</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>beijing-thumbnail</x:v>
@@ -1503,7 +1518,7 @@
         <x:v>beijing-detail-normal</x:v>
       </x:c>
       <x:c r="M8" s="10" t="str">
-        <x:v>{"cityId":"beijing","name":"北京","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"beijing-thumbnail","light":{"mask":"beijing-light-mask","normal":"beijing-light-normal"},"standard":{"mask":"beijing-standard-mask","normal":"beijing-standard-normal"},"detail":{"mask":"beijing-detail-mask","normal":"beijing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"beijing","name":"北京","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"beijing-thumbnail","light":{"mask":"beijing-light-mask","normal":"beijing-light-normal"},"standard":{"mask":"beijing-standard-mask","normal":"beijing-standard-normal"},"detail":{"mask":"beijing-detail-mask","normal":"beijing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
@@ -1517,10 +1532,10 @@
         <x:v>南京</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
         <x:v>nanjing-thumbnail</x:v>
@@ -1544,7 +1559,7 @@
         <x:v>nanjing-detail-normal</x:v>
       </x:c>
       <x:c r="M9" s="11" t="str">
-        <x:v>{"cityId":"nanjing","name":"南京","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"nanjing-thumbnail","light":{"mask":"nanjing-light-mask","normal":"nanjing-light-normal"},"standard":{"mask":"nanjing-standard-mask","normal":"nanjing-standard-normal"},"detail":{"mask":"nanjing-detail-mask","normal":"nanjing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"nanjing","name":"南京","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"nanjing-thumbnail","light":{"mask":"nanjing-light-mask","normal":"nanjing-light-normal"},"standard":{"mask":"nanjing-standard-mask","normal":"nanjing-standard-normal"},"detail":{"mask":"nanjing-detail-mask","normal":"nanjing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
@@ -1558,10 +1573,10 @@
         <x:v>南昌</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
         <x:v>nanchang-thumbnail</x:v>
@@ -1585,7 +1600,7 @@
         <x:v>nanchang-detail-normal</x:v>
       </x:c>
       <x:c r="M10" s="10" t="str">
-        <x:v>{"cityId":"nanchang","name":"南昌","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"nanchang-thumbnail","light":{"mask":"nanchang-light-mask","normal":"nanchang-light-normal"},"standard":{"mask":"nanchang-standard-mask","normal":"nanchang-standard-normal"},"detail":{"mask":"nanchang-detail-mask","normal":"nanchang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"nanchang","name":"南昌","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"nanchang-thumbnail","light":{"mask":"nanchang-light-mask","normal":"nanchang-light-normal"},"standard":{"mask":"nanchang-standard-mask","normal":"nanchang-standard-normal"},"detail":{"mask":"nanchang-detail-mask","normal":"nanchang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
@@ -1599,10 +1614,10 @@
         <x:v>厦门</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
         <x:v>xiamen-thumbnail</x:v>
@@ -1626,7 +1641,7 @@
         <x:v>xiamen-detail-normal</x:v>
       </x:c>
       <x:c r="M11" s="11" t="str">
-        <x:v>{"cityId":"xiamen","name":"厦门","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"xiamen-thumbnail","light":{"mask":"xiamen-light-mask","normal":"xiamen-light-normal"},"standard":{"mask":"xiamen-standard-mask","normal":"xiamen-standard-normal"},"detail":{"mask":"xiamen-detail-mask","normal":"xiamen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"xiamen","name":"厦门","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"xiamen-thumbnail","light":{"mask":"xiamen-light-mask","normal":"xiamen-light-normal"},"standard":{"mask":"xiamen-standard-mask","normal":"xiamen-standard-normal"},"detail":{"mask":"xiamen-detail-mask","normal":"xiamen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
@@ -1640,10 +1655,10 @@
         <x:v>呼和浩特</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
         <x:v>hohhot-thumbnail</x:v>
@@ -1667,7 +1682,7 @@
         <x:v>hohhot-detail-normal</x:v>
       </x:c>
       <x:c r="M12" s="10" t="str">
-        <x:v>{"cityId":"hohhot","name":"呼和浩特","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"hohhot-thumbnail","light":{"mask":"hohhot-light-mask","normal":"hohhot-light-normal"},"standard":{"mask":"hohhot-standard-mask","normal":"hohhot-standard-normal"},"detail":{"mask":"hohhot-detail-mask","normal":"hohhot-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"hohhot","name":"呼和浩特","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"hohhot-thumbnail","light":{"mask":"hohhot-light-mask","normal":"hohhot-light-normal"},"standard":{"mask":"hohhot-standard-mask","normal":"hohhot-standard-normal"},"detail":{"mask":"hohhot-detail-mask","normal":"hohhot-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
@@ -1681,10 +1696,10 @@
         <x:v>哈尔滨</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
         <x:v>harbin-thumbnail</x:v>
@@ -1708,7 +1723,7 @@
         <x:v>harbin-detail-normal</x:v>
       </x:c>
       <x:c r="M13" s="11" t="str">
-        <x:v>{"cityId":"harbin","name":"哈尔滨","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"harbin-thumbnail","light":{"mask":"harbin-light-mask","normal":"harbin-light-normal"},"standard":{"mask":"harbin-standard-mask","normal":"harbin-standard-normal"},"detail":{"mask":"harbin-detail-mask","normal":"harbin-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"harbin","name":"哈尔滨","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"harbin-thumbnail","light":{"mask":"harbin-light-mask","normal":"harbin-light-normal"},"standard":{"mask":"harbin-standard-mask","normal":"harbin-standard-normal"},"detail":{"mask":"harbin-detail-mask","normal":"harbin-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1722,10 +1737,10 @@
         <x:v>天津</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>tianjin-thumbnail</x:v>
@@ -1749,7 +1764,7 @@
         <x:v>tianjin-detail-normal</x:v>
       </x:c>
       <x:c r="M14" s="10" t="str">
-        <x:v>{"cityId":"tianjin","name":"天津","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"tianjin-thumbnail","light":{"mask":"tianjin-light-mask","normal":"tianjin-light-normal"},"standard":{"mask":"tianjin-standard-mask","normal":"tianjin-standard-normal"},"detail":{"mask":"tianjin-detail-mask","normal":"tianjin-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"tianjin","name":"天津","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"tianjin-thumbnail","light":{"mask":"tianjin-light-mask","normal":"tianjin-light-normal"},"standard":{"mask":"tianjin-standard-mask","normal":"tianjin-standard-normal"},"detail":{"mask":"tianjin-detail-mask","normal":"tianjin-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
@@ -1763,10 +1778,10 @@
         <x:v>太原</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
         <x:v>taiyuan-thumbnail</x:v>
@@ -1790,7 +1805,7 @@
         <x:v>taiyuan-detail-normal</x:v>
       </x:c>
       <x:c r="M15" s="11" t="str">
-        <x:v>{"cityId":"taiyuan","name":"太原","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"taiyuan-thumbnail","light":{"mask":"taiyuan-light-mask","normal":"taiyuan-light-normal"},"standard":{"mask":"taiyuan-standard-mask","normal":"taiyuan-standard-normal"},"detail":{"mask":"taiyuan-detail-mask","normal":"taiyuan-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"taiyuan","name":"太原","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"taiyuan-thumbnail","light":{"mask":"taiyuan-light-mask","normal":"taiyuan-light-normal"},"standard":{"mask":"taiyuan-standard-mask","normal":"taiyuan-standard-normal"},"detail":{"mask":"taiyuan-detail-mask","normal":"taiyuan-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
@@ -1804,10 +1819,10 @@
         <x:v>广州</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
         <x:v>guangzhou-thumbnail</x:v>
@@ -1831,7 +1846,7 @@
         <x:v>guangzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M16" s="10" t="str">
-        <x:v>{"cityId":"guangzhou","name":"广州","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"guangzhou-thumbnail","light":{"mask":"guangzhou-light-mask","normal":"guangzhou-light-normal"},"standard":{"mask":"guangzhou-standard-mask","normal":"guangzhou-standard-normal"},"detail":{"mask":"guangzhou-detail-mask","normal":"guangzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"guangzhou","name":"广州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"guangzhou-thumbnail","light":{"mask":"guangzhou-light-mask","normal":"guangzhou-light-normal"},"standard":{"mask":"guangzhou-standard-mask","normal":"guangzhou-standard-normal"},"detail":{"mask":"guangzhou-detail-mask","normal":"guangzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
@@ -1845,10 +1860,10 @@
         <x:v>成都</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E17" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
         <x:v>chengdu-thumbnail</x:v>
@@ -1872,7 +1887,7 @@
         <x:v>chengdu-detail-normal</x:v>
       </x:c>
       <x:c r="M17" s="11" t="str">
-        <x:v>{"cityId":"chengdu","name":"成都","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"chengdu-thumbnail","light":{"mask":"chengdu-light-mask","normal":"chengdu-light-normal"},"standard":{"mask":"chengdu-standard-mask","normal":"chengdu-standard-normal"},"detail":{"mask":"chengdu-detail-mask","normal":"chengdu-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"chengdu","name":"成都","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"chengdu-thumbnail","light":{"mask":"chengdu-light-mask","normal":"chengdu-light-normal"},"standard":{"mask":"chengdu-standard-mask","normal":"chengdu-standard-normal"},"detail":{"mask":"chengdu-detail-mask","normal":"chengdu-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -1886,10 +1901,10 @@
         <x:v>景德镇</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E18" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F18" s="10" t="str">
         <x:v>jingdezhen-thumbnail</x:v>
@@ -1913,7 +1928,7 @@
         <x:v>jingdezhen-detail-normal</x:v>
       </x:c>
       <x:c r="M18" s="10" t="str">
-        <x:v>{"cityId":"jingdezhen","name":"景德镇","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"jingdezhen-thumbnail","light":{"mask":"jingdezhen-light-mask","normal":"jingdezhen-light-normal"},"standard":{"mask":"jingdezhen-standard-mask","normal":"jingdezhen-standard-normal"},"detail":{"mask":"jingdezhen-detail-mask","normal":"jingdezhen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"jingdezhen","name":"景德镇","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"jingdezhen-thumbnail","light":{"mask":"jingdezhen-light-mask","normal":"jingdezhen-light-normal"},"standard":{"mask":"jingdezhen-standard-mask","normal":"jingdezhen-standard-normal"},"detail":{"mask":"jingdezhen-detail-mask","normal":"jingdezhen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -1927,10 +1942,10 @@
         <x:v>杭州</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E19" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F19" s="11" t="str">
         <x:v>hangzhou-thumbnail</x:v>
@@ -1954,7 +1969,7 @@
         <x:v>hangzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M19" s="11" t="str">
-        <x:v>{"cityId":"hangzhou","name":"杭州","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"hangzhou-thumbnail","light":{"mask":"hangzhou-light-mask","normal":"hangzhou-light-normal"},"standard":{"mask":"hangzhou-standard-mask","normal":"hangzhou-standard-normal"},"detail":{"mask":"hangzhou-detail-mask","normal":"hangzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"hangzhou","name":"杭州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"hangzhou-thumbnail","light":{"mask":"hangzhou-light-mask","normal":"hangzhou-light-normal"},"standard":{"mask":"hangzhou-standard-mask","normal":"hangzhou-standard-normal"},"detail":{"mask":"hangzhou-detail-mask","normal":"hangzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -1968,10 +1983,10 @@
         <x:v>武汉</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E20" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F20" s="10" t="str">
         <x:v>wuhan-thumbnail</x:v>
@@ -1995,7 +2010,7 @@
         <x:v>wuhan-detail-normal</x:v>
       </x:c>
       <x:c r="M20" s="10" t="str">
-        <x:v>{"cityId":"wuhan","name":"武汉","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"wuhan-thumbnail","light":{"mask":"wuhan-light-mask","normal":"wuhan-light-normal"},"standard":{"mask":"wuhan-standard-mask","normal":"wuhan-standard-normal"},"detail":{"mask":"wuhan-detail-mask","normal":"wuhan-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"wuhan","name":"武汉","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"wuhan-thumbnail","light":{"mask":"wuhan-light-mask","normal":"wuhan-light-normal"},"standard":{"mask":"wuhan-standard-mask","normal":"wuhan-standard-normal"},"detail":{"mask":"wuhan-detail-mask","normal":"wuhan-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -2009,10 +2024,10 @@
         <x:v>沈阳</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
         <x:v>shenyang-thumbnail</x:v>
@@ -2036,7 +2051,7 @@
         <x:v>shenyang-detail-normal</x:v>
       </x:c>
       <x:c r="M21" s="11" t="str">
-        <x:v>{"cityId":"shenyang","name":"沈阳","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"shenyang-thumbnail","light":{"mask":"shenyang-light-mask","normal":"shenyang-light-normal"},"standard":{"mask":"shenyang-standard-mask","normal":"shenyang-standard-normal"},"detail":{"mask":"shenyang-detail-mask","normal":"shenyang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shenyang","name":"沈阳","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shenyang-thumbnail","light":{"mask":"shenyang-light-mask","normal":"shenyang-light-normal"},"standard":{"mask":"shenyang-standard-mask","normal":"shenyang-standard-normal"},"detail":{"mask":"shenyang-detail-mask","normal":"shenyang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -2050,10 +2065,10 @@
         <x:v>深圳</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
         <x:v>shenzhen-thumbnail</x:v>
@@ -2077,7 +2092,7 @@
         <x:v>shenzhen-detail-normal</x:v>
       </x:c>
       <x:c r="M22" s="10" t="str">
-        <x:v>{"cityId":"shenzhen","name":"深圳","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"shenzhen-thumbnail","light":{"mask":"shenzhen-light-mask","normal":"shenzhen-light-normal"},"standard":{"mask":"shenzhen-standard-mask","normal":"shenzhen-standard-normal"},"detail":{"mask":"shenzhen-detail-mask","normal":"shenzhen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shenzhen","name":"深圳","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shenzhen-thumbnail","light":{"mask":"shenzhen-light-mask","normal":"shenzhen-light-normal"},"standard":{"mask":"shenzhen-standard-mask","normal":"shenzhen-standard-normal"},"detail":{"mask":"shenzhen-detail-mask","normal":"shenzhen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -2091,10 +2106,10 @@
         <x:v>石家庄</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E23" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F23" s="11" t="str">
         <x:v>shijiazhuang-thumbnail</x:v>
@@ -2118,7 +2133,7 @@
         <x:v>shijiazhuang-detail-normal</x:v>
       </x:c>
       <x:c r="M23" s="11" t="str">
-        <x:v>{"cityId":"shijiazhuang","name":"石家庄","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"shijiazhuang-thumbnail","light":{"mask":"shijiazhuang-light-mask","normal":"shijiazhuang-light-normal"},"standard":{"mask":"shijiazhuang-standard-mask","normal":"shijiazhuang-standard-normal"},"detail":{"mask":"shijiazhuang-detail-mask","normal":"shijiazhuang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shijiazhuang","name":"石家庄","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shijiazhuang-thumbnail","light":{"mask":"shijiazhuang-light-mask","normal":"shijiazhuang-light-normal"},"standard":{"mask":"shijiazhuang-standard-mask","normal":"shijiazhuang-standard-normal"},"detail":{"mask":"shijiazhuang-detail-mask","normal":"shijiazhuang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
@@ -2132,10 +2147,10 @@
         <x:v>西安</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
         <x:v>xian-thumbnail</x:v>
@@ -2159,7 +2174,7 @@
         <x:v>xian-detail-normal</x:v>
       </x:c>
       <x:c r="M24" s="10" t="str">
-        <x:v>{"cityId":"xian","name":"西安","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"xian-thumbnail","light":{"mask":"xian-light-mask","normal":"xian-light-normal"},"standard":{"mask":"xian-standard-mask","normal":"xian-standard-normal"},"detail":{"mask":"xian-detail-mask","normal":"xian-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"xian","name":"西安","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"xian-thumbnail","light":{"mask":"xian-light-mask","normal":"xian-light-normal"},"standard":{"mask":"xian-standard-mask","normal":"xian-standard-normal"},"detail":{"mask":"xian-detail-mask","normal":"xian-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
@@ -2173,10 +2188,10 @@
         <x:v>郑州</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E25" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F25" s="11" t="str">
         <x:v>zhengzhou-thumbnail</x:v>
@@ -2200,7 +2215,7 @@
         <x:v>zhengzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M25" s="11" t="str">
-        <x:v>{"cityId":"zhengzhou","name":"郑州","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"zhengzhou-thumbnail","light":{"mask":"zhengzhou-light-mask","normal":"zhengzhou-light-normal"},"standard":{"mask":"zhengzhou-standard-mask","normal":"zhengzhou-standard-normal"},"detail":{"mask":"zhengzhou-detail-mask","normal":"zhengzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"zhengzhou","name":"郑州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"zhengzhou-thumbnail","light":{"mask":"zhengzhou-light-mask","normal":"zhengzhou-light-normal"},"standard":{"mask":"zhengzhou-standard-mask","normal":"zhengzhou-standard-normal"},"detail":{"mask":"zhengzhou-detail-mask","normal":"zhengzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
@@ -2214,10 +2229,10 @@
         <x:v>重庆</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F26" s="10" t="str">
         <x:v>chongqing-thumbnail</x:v>
@@ -2241,7 +2256,7 @@
         <x:v>chongqing-detail-normal</x:v>
       </x:c>
       <x:c r="M26" s="10" t="str">
-        <x:v>{"cityId":"chongqing","name":"重庆","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"chongqing-thumbnail","light":{"mask":"chongqing-light-mask","normal":"chongqing-light-normal"},"standard":{"mask":"chongqing-standard-mask","normal":"chongqing-standard-normal"},"detail":{"mask":"chongqing-detail-mask","normal":"chongqing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"chongqing","name":"重庆","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"chongqing-thumbnail","light":{"mask":"chongqing-light-mask","normal":"chongqing-light-normal"},"standard":{"mask":"chongqing-standard-mask","normal":"chongqing-standard-normal"},"detail":{"mask":"chongqing-detail-mask","normal":"chongqing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -2255,10 +2270,10 @@
         <x:v>长春</x:v>
       </x:c>
       <x:c r="D27" s="11" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E27" s="11" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F27" s="11" t="str">
         <x:v>changchun-thumbnail</x:v>
@@ -2282,7 +2297,7 @@
         <x:v>changchun-detail-normal</x:v>
       </x:c>
       <x:c r="M27" s="11" t="str">
-        <x:v>{"cityId":"changchun","name":"长春","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"changchun-thumbnail","light":{"mask":"changchun-light-mask","normal":"changchun-light-normal"},"standard":{"mask":"changchun-standard-mask","normal":"changchun-standard-normal"},"detail":{"mask":"changchun-detail-mask","normal":"changchun-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"changchun","name":"长春","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"changchun-thumbnail","light":{"mask":"changchun-light-mask","normal":"changchun-light-normal"},"standard":{"mask":"changchun-standard-mask","normal":"changchun-standard-normal"},"detail":{"mask":"changchun-detail-mask","normal":"changchun-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -2296,10 +2311,10 @@
         <x:v>青岛</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>v7-2</x:v>
+        <x:v>v7-3</x:v>
       </x:c>
       <x:c r="E28" s="10" t="str">
-        <x:v>releases/v7-2/manifest-c3af02ef5468edcb.json</x:v>
+        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
       </x:c>
       <x:c r="F28" s="10" t="str">
         <x:v>qingdao-thumbnail</x:v>
@@ -2323,13 +2338,13 @@
         <x:v>qingdao-detail-normal</x:v>
       </x:c>
       <x:c r="M28" s="10" t="str">
-        <x:v>{"cityId":"qingdao","name":"青岛","resourceReleaseId":"v7-2","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-2/manifest-c3af02ef5468edcb.json","resourceIds":{"thumbnail":"qingdao-thumbnail","light":{"mask":"qingdao-light-mask","normal":"qingdao-light-normal"},"standard":{"mask":"qingdao-standard-mask","normal":"qingdao-standard-normal"},"detail":{"mask":"qingdao-detail-mask","normal":"qingdao-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"qingdao","name":"青岛","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"qingdao-thumbnail","light":{"mask":"qingdao-light-mask","normal":"qingdao-light-normal"},"standard":{"mask":"qingdao-standard-mask","normal":"qingdao-standard-normal"},"detail":{"mask":"qingdao-detail-mask","normal":"qingdao-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9655adfa6bd34a11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73ce3e95983e4d98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2390,7 +2405,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2699,7 +2714,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f0f0709ca2f470d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2333119161614b6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2742,7 +2757,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3106,7 +3121,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63bb2c8e128b4cd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4989efc715743a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3149,7 +3164,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3195,7 +3210,7 @@
         <x:v>编码与加载</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="45" customHeight="1">
+    <x:row r="6" ht="65" customHeight="1">
       <x:c r="A6" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -3209,19 +3224,19 @@
         <x:v>slogan-open</x:v>
       </x:c>
       <x:c r="E6" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F6" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G6" s="10" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H6" s="10" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="45" customHeight="1">
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="65" customHeight="1">
       <x:c r="A7" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -3235,19 +3250,19 @@
         <x:v>slogan-innovation</x:v>
       </x:c>
       <x:c r="E7" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F7" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="45" customHeight="1">
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="65" customHeight="1">
       <x:c r="A8" s="14" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -3261,19 +3276,19 @@
         <x:v>slogan-cooperation</x:v>
       </x:c>
       <x:c r="E8" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F8" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G8" s="10" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="45" customHeight="1">
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="65" customHeight="1">
       <x:c r="A9" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -3287,19 +3302,19 @@
         <x:v>slogan-sharing</x:v>
       </x:c>
       <x:c r="E9" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F9" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="45" customHeight="1">
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="65" customHeight="1">
       <x:c r="A10" s="14" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -3313,19 +3328,19 @@
         <x:v>slogan-together</x:v>
       </x:c>
       <x:c r="E10" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F10" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="45" customHeight="1">
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="65" customHeight="1">
       <x:c r="A11" s="16" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -3339,22 +3354,22 @@
         <x:v>slogan-ocean</x:v>
       </x:c>
       <x:c r="E11" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="F11" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str">
-        <x:v>[0.774658203125,0.3881099270891756,0.070556640625,0.5238362310712282]</x:v>
+        <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>WebP线性R8；左下UV原点；4px护边；六组首屏解码上传；运行时不渲染SVG</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2be16e1cffc54708"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ed795bf71f94bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3433,7 +3448,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.1 / v7-2 / ec6f9bb0b606 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7474,7 +7489,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J69" s="16" t="n">
-        <x:v>46200</x:v>
+        <x:v>46286</x:v>
       </x:c>
       <x:c r="K69" s="16" t="n">
         <x:v>913408</x:v>
@@ -7492,19 +7507,19 @@
         <x:v>1217878</x:v>
       </x:c>
       <x:c r="P69" s="11" t="str">
-        <x:v>../v7-1/assets/xiamen-light-mask-65634b05877a400b.webp</x:v>
+        <x:v>assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
       </x:c>
       <x:c r="Q69" s="11" t="str">
-        <x:v>releases/v7-1/assets/xiamen-light-mask-65634b05877a400b.webp</x:v>
+        <x:v>releases/v7-3/assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
       </x:c>
       <x:c r="R69" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/xiamen-light-mask-65634b05877a400b.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
       </x:c>
       <x:c r="S69" s="11" t="str">
-        <x:v>65634b05877a400b30e0782c5c28befea899bc3a81e60504b3b7b21c7ad21d0c</x:v>
+        <x:v>43538debb37bd8265ff918e4e42f28c77124e94e95159ba5bc80f143c361d6cf</x:v>
       </x:c>
       <x:c r="T69" s="11" t="str">
-        <x:v>6a1e5d9bf6267ad3566279b74cf4a48244dfe69a4ea6e331ffb400b82eb12c7f</x:v>
+        <x:v>ee68b1a111837996d96fba0774a432938cabf682358fc288787ae1a05991a1b6</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
@@ -7598,7 +7613,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J71" s="16" t="n">
-        <x:v>115008</x:v>
+        <x:v>115220</x:v>
       </x:c>
       <x:c r="K71" s="16" t="n">
         <x:v>3653632</x:v>
@@ -7616,19 +7631,19 @@
         <x:v>4871510</x:v>
       </x:c>
       <x:c r="P71" s="11" t="str">
-        <x:v>../v7-1/assets/xiamen-standard-mask-4d85ba0b13a08bfb.webp</x:v>
+        <x:v>assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
       </x:c>
       <x:c r="Q71" s="11" t="str">
-        <x:v>releases/v7-1/assets/xiamen-standard-mask-4d85ba0b13a08bfb.webp</x:v>
+        <x:v>releases/v7-3/assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
       </x:c>
       <x:c r="R71" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/xiamen-standard-mask-4d85ba0b13a08bfb.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
       </x:c>
       <x:c r="S71" s="11" t="str">
-        <x:v>4d85ba0b13a08bfb46becb80883c7e2f7c7f2134ac2f795ac80658760a2518d9</x:v>
+        <x:v>403c47be25586d7a21c449c260d4f035e121746385c468e4a2f82843c91d92b9</x:v>
       </x:c>
       <x:c r="T71" s="11" t="str">
-        <x:v>6a1e5d9bf6267ad3566279b74cf4a48244dfe69a4ea6e331ffb400b82eb12c7f</x:v>
+        <x:v>f68612cebb63411e052c72bc695c78a51e9ef404a5da45aab71d4e4ac9de6d30</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
@@ -7722,7 +7737,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J73" s="16" t="n">
-        <x:v>198370</x:v>
+        <x:v>198398</x:v>
       </x:c>
       <x:c r="K73" s="16" t="n">
         <x:v>14606336</x:v>
@@ -7740,19 +7755,19 @@
         <x:v>19475115</x:v>
       </x:c>
       <x:c r="P73" s="11" t="str">
-        <x:v>../v7-1/assets/xiamen-detail-mask-6a1e5d9bf6267ad3.webp</x:v>
+        <x:v>assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
       </x:c>
       <x:c r="Q73" s="11" t="str">
-        <x:v>releases/v7-1/assets/xiamen-detail-mask-6a1e5d9bf6267ad3.webp</x:v>
+        <x:v>releases/v7-3/assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
       </x:c>
       <x:c r="R73" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/xiamen-detail-mask-6a1e5d9bf6267ad3.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
       </x:c>
       <x:c r="S73" s="11" t="str">
-        <x:v>6a1e5d9bf6267ad3566279b74cf4a48244dfe69a4ea6e331ffb400b82eb12c7f</x:v>
+        <x:v>7e7d2ac8b97d19f8cb09377952d34074d35422fda354872913e8e765af287549</x:v>
       </x:c>
       <x:c r="T73" s="11" t="str">
-        <x:v>6a1e5d9bf6267ad3566279b74cf4a48244dfe69a4ea6e331ffb400b82eb12c7f</x:v>
+        <x:v>72647e9af88e0e15fb4fe898b0f8a9877c2d5c4d8355c669b635433811f2c484</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
@@ -13116,7 +13131,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J160" s="14" t="n">
-        <x:v>49984</x:v>
+        <x:v>50280</x:v>
       </x:c>
       <x:c r="K160" s="14" t="n">
         <x:v>913408</x:v>
@@ -13134,19 +13149,19 @@
         <x:v>1217878</x:v>
       </x:c>
       <x:c r="P160" s="10" t="str">
-        <x:v>assets/xian-light-mask-02a6808d8532b8af.webp</x:v>
+        <x:v>assets/xian-light-mask-c5024f591539dc71.webp</x:v>
       </x:c>
       <x:c r="Q160" s="10" t="str">
-        <x:v>releases/v7-2/assets/xian-light-mask-02a6808d8532b8af.webp</x:v>
+        <x:v>releases/v7-3/assets/xian-light-mask-c5024f591539dc71.webp</x:v>
       </x:c>
       <x:c r="R160" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-2/assets/xian-light-mask-02a6808d8532b8af.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xian-light-mask-c5024f591539dc71.webp</x:v>
       </x:c>
       <x:c r="S160" s="10" t="str">
-        <x:v>02a6808d8532b8af51e4534af62fe125e6c398470fd8435bbfa8a3196e658816</x:v>
+        <x:v>c5024f591539dc7123cac1cf19e119bf146d59fcb5b249dd3e581ec1c1c3a89e</x:v>
       </x:c>
       <x:c r="T160" s="10" t="str">
-        <x:v>ae6038888c4eb92d755966e9a2a8e6a9527b26f71a199be42667fd1546c4cd28</x:v>
+        <x:v>3ac72d0b8185245a2ba28118e5c3b6029ccc11dbad55b65a2073d0a1c98fbedb</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="42" customHeight="1">
@@ -13240,7 +13255,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J162" s="14" t="n">
-        <x:v>132694</x:v>
+        <x:v>132670</x:v>
       </x:c>
       <x:c r="K162" s="14" t="n">
         <x:v>3653632</x:v>
@@ -13258,19 +13273,19 @@
         <x:v>4871510</x:v>
       </x:c>
       <x:c r="P162" s="10" t="str">
-        <x:v>assets/xian-standard-mask-547ec8ef8b249bce.webp</x:v>
+        <x:v>assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
       </x:c>
       <x:c r="Q162" s="10" t="str">
-        <x:v>releases/v7-2/assets/xian-standard-mask-547ec8ef8b249bce.webp</x:v>
+        <x:v>releases/v7-3/assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
       </x:c>
       <x:c r="R162" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-2/assets/xian-standard-mask-547ec8ef8b249bce.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
       </x:c>
       <x:c r="S162" s="10" t="str">
-        <x:v>547ec8ef8b249bce47baa9a35fdea3f65921e870f51d5e5f369d412bdb8a2bba</x:v>
+        <x:v>6765eb28884cba73b5aeab4fb4a93bbc8d6ef3478c2f40e13ac5341e8374a071</x:v>
       </x:c>
       <x:c r="T162" s="10" t="str">
-        <x:v>ae6038888c4eb92d755966e9a2a8e6a9527b26f71a199be42667fd1546c4cd28</x:v>
+        <x:v>25823c1deb22e635369d3415670304ca60e748e4974fb19b74a92237e0f1d207</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="42" customHeight="1">
@@ -13364,7 +13379,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="J164" s="14" t="n">
-        <x:v>225744</x:v>
+        <x:v>225564</x:v>
       </x:c>
       <x:c r="K164" s="14" t="n">
         <x:v>14606336</x:v>
@@ -13382,19 +13397,19 @@
         <x:v>19475115</x:v>
       </x:c>
       <x:c r="P164" s="10" t="str">
-        <x:v>assets/xian-detail-mask-cd07e2cae76c63a6.webp</x:v>
+        <x:v>assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
       </x:c>
       <x:c r="Q164" s="10" t="str">
-        <x:v>releases/v7-2/assets/xian-detail-mask-cd07e2cae76c63a6.webp</x:v>
+        <x:v>releases/v7-3/assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
       </x:c>
       <x:c r="R164" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-2/assets/xian-detail-mask-cd07e2cae76c63a6.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
       </x:c>
       <x:c r="S164" s="10" t="str">
-        <x:v>cd07e2cae76c63a69d83bf8f441b536dc21ac0f993dd9e0be745f85823017721</x:v>
+        <x:v>2fec346956d39c3bcc25967e818c297c9927383fcfc05ce6e33418328a563fc2</x:v>
       </x:c>
       <x:c r="T164" s="10" t="str">
-        <x:v>ae6038888c4eb92d755966e9a2a8e6a9527b26f71a199be42667fd1546c4cd28</x:v>
+        <x:v>3d4926de6a16340bffa1d2fd2389f10863d78e3b743d82d6fe0468f9237fcfb8</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="42" customHeight="1">
@@ -15215,46 +15230,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G194" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H194" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I194" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J194" s="14" t="n">
-        <x:v>17470</x:v>
+        <x:v>13680</x:v>
       </x:c>
       <x:c r="K194" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L194" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M194" s="10" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N194" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O194" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P194" s="10" t="str">
-        <x:v>../v7-1/assets/slogan-open-6180ec934a95c4d5.webp</x:v>
+        <x:v>assets/slogan-open-d0dc0df725a844be.webp</x:v>
       </x:c>
       <x:c r="Q194" s="10" t="str">
-        <x:v>releases/v7-1/assets/slogan-open-6180ec934a95c4d5.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-open-d0dc0df725a844be.webp</x:v>
       </x:c>
       <x:c r="R194" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-open-6180ec934a95c4d5.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-open-d0dc0df725a844be.webp</x:v>
       </x:c>
       <x:c r="S194" s="10" t="str">
-        <x:v>6180ec934a95c4d53387c6a3843dc8134e52e2e9b69db88894e892cbec6988fd</x:v>
+        <x:v>d0dc0df725a844be17183846ee7efe114fcc3f1009a0efaee703254378d40126</x:v>
       </x:c>
       <x:c r="T194" s="10" t="str">
-        <x:v>8264d0763a1afdf47c7c70d00b3c8f694dd913af270d9b408c1bd619ee34109e</x:v>
+        <x:v>4bb4fc55916758d5253a91cf40d8a62474733ff293045e4c4ae9e397be8df178</x:v>
       </x:c>
     </x:row>
     <x:row r="195" ht="42" customHeight="1">
@@ -15277,46 +15292,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G195" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H195" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I195" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J195" s="16" t="n">
-        <x:v>18558</x:v>
+        <x:v>15024</x:v>
       </x:c>
       <x:c r="K195" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L195" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M195" s="11" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N195" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O195" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P195" s="11" t="str">
-        <x:v>../v7-1/assets/slogan-innovation-23940d813f68f7f2.webp</x:v>
+        <x:v>assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
       </x:c>
       <x:c r="Q195" s="11" t="str">
-        <x:v>releases/v7-1/assets/slogan-innovation-23940d813f68f7f2.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
       </x:c>
       <x:c r="R195" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-innovation-23940d813f68f7f2.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
       </x:c>
       <x:c r="S195" s="11" t="str">
-        <x:v>23940d813f68f7f2d3e715630a944abb18f74d319b2a0cd78a6acb1fcae60e10</x:v>
+        <x:v>0c31d18458db52dd67f18cb0a7a94e82a0c5e934f4b629664994b37075798556</x:v>
       </x:c>
       <x:c r="T195" s="11" t="str">
-        <x:v>afdb28c9490033748ba6d13adedbb125163d5dce13de832241a457668363ba2e</x:v>
+        <x:v>d9f0655b57e762ccb1bc2d8fabda1e2e10169d750927da929ca3a29165ede2c8</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="42" customHeight="1">
@@ -15339,46 +15354,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G196" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H196" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I196" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J196" s="14" t="n">
-        <x:v>17800</x:v>
+        <x:v>12632</x:v>
       </x:c>
       <x:c r="K196" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L196" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M196" s="10" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N196" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O196" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P196" s="10" t="str">
-        <x:v>../v7-1/assets/slogan-cooperation-7c0daa11ce6fefa6.webp</x:v>
+        <x:v>assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
       </x:c>
       <x:c r="Q196" s="10" t="str">
-        <x:v>releases/v7-1/assets/slogan-cooperation-7c0daa11ce6fefa6.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
       </x:c>
       <x:c r="R196" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-cooperation-7c0daa11ce6fefa6.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
       </x:c>
       <x:c r="S196" s="10" t="str">
-        <x:v>7c0daa11ce6fefa68714604c135774448962e1532b3d4e5d67c86925b6140eda</x:v>
+        <x:v>e2c5f6b534591635051fa826c08b3b55e13bbecb42e6a2e2a25c5fe931181fe9</x:v>
       </x:c>
       <x:c r="T196" s="10" t="str">
-        <x:v>21de4a3f69e3e253df36c5edae336816ccaf7ef70bc30ff09d1ea9940dc01305</x:v>
+        <x:v>2999d4de9baa2231d20e6ba096a3026940b1f21588704f88ed86effd5ff4c693</x:v>
       </x:c>
     </x:row>
     <x:row r="197" ht="42" customHeight="1">
@@ -15401,46 +15416,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G197" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H197" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I197" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J197" s="16" t="n">
-        <x:v>16856</x:v>
+        <x:v>11912</x:v>
       </x:c>
       <x:c r="K197" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L197" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M197" s="11" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N197" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O197" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P197" s="11" t="str">
-        <x:v>../v7-1/assets/slogan-sharing-4e868028d70e2abb.webp</x:v>
+        <x:v>assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
       </x:c>
       <x:c r="Q197" s="11" t="str">
-        <x:v>releases/v7-1/assets/slogan-sharing-4e868028d70e2abb.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
       </x:c>
       <x:c r="R197" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-sharing-4e868028d70e2abb.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
       </x:c>
       <x:c r="S197" s="11" t="str">
-        <x:v>4e868028d70e2abb26b69bcca4942271b6823c10d92f4efa893c471fd283114f</x:v>
+        <x:v>7d2d7bf570a46ce8dc758724cb6981d9339a8087cc3b8b0d47e37784310369a2</x:v>
       </x:c>
       <x:c r="T197" s="11" t="str">
-        <x:v>f5407c1f9a5495636f99dc1edb5985301257ebf15f070e5c47956868a9ccf571</x:v>
+        <x:v>b088533e404deb956a0455a9f7651deb7e1dfa87924b32826f07a6c77a999466</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="42" customHeight="1">
@@ -15463,46 +15478,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G198" s="14" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H198" s="14" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I198" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J198" s="14" t="n">
-        <x:v>16860</x:v>
+        <x:v>11890</x:v>
       </x:c>
       <x:c r="K198" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L198" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M198" s="10" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N198" s="14" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O198" s="14" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P198" s="10" t="str">
-        <x:v>../v7-1/assets/slogan-together-a77c25b8f7293b3e.webp</x:v>
+        <x:v>assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
       </x:c>
       <x:c r="Q198" s="10" t="str">
-        <x:v>releases/v7-1/assets/slogan-together-a77c25b8f7293b3e.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
       </x:c>
       <x:c r="R198" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-together-a77c25b8f7293b3e.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
       </x:c>
       <x:c r="S198" s="10" t="str">
-        <x:v>a77c25b8f7293b3ed06a879cfaf5a41f6e2a84a4e19bd92d138ee1d5b6f170f7</x:v>
+        <x:v>7e3a2c69d745a00f9d027f9add8a24fb9d5406d9cf9771c7951214a057c00d2b</x:v>
       </x:c>
       <x:c r="T198" s="10" t="str">
-        <x:v>86e553e8af7cb34a9004cf7ed806992c21e507708563a997b5987fdf7cb28fc5</x:v>
+        <x:v>103598f5e5ce7db1538f361e5661b7ee78c8f35365dfd615bd907387d25b7024</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="42" customHeight="1">
@@ -15525,46 +15540,46 @@
         <x:v>linear</x:v>
       </x:c>
       <x:c r="G199" s="16" t="n">
-        <x:v>289</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="H199" s="16" t="n">
-        <x:v>934</x:v>
+        <x:v>936</x:v>
       </x:c>
       <x:c r="I199" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J199" s="16" t="n">
-        <x:v>19178</x:v>
+        <x:v>15404</x:v>
       </x:c>
       <x:c r="K199" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="L199" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="M199" s="11" t="str">
         <x:v>R8</x:v>
       </x:c>
       <x:c r="N199" s="16" t="n">
-        <x:v>269926</x:v>
+        <x:v>269568</x:v>
       </x:c>
       <x:c r="O199" s="16" t="n">
-        <x:v>359902</x:v>
+        <x:v>359424</x:v>
       </x:c>
       <x:c r="P199" s="11" t="str">
-        <x:v>../v7-1/assets/slogan-ocean-d480bfd4c681c6c2.webp</x:v>
+        <x:v>assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
       </x:c>
       <x:c r="Q199" s="11" t="str">
-        <x:v>releases/v7-1/assets/slogan-ocean-d480bfd4c681c6c2.webp</x:v>
+        <x:v>releases/v7-3/assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
       </x:c>
       <x:c r="R199" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/slogan-ocean-d480bfd4c681c6c2.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-3/assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
       </x:c>
       <x:c r="S199" s="11" t="str">
-        <x:v>d480bfd4c681c6c29da216d1976df7ca8b3246c968227310d7d959786ee2fd26</x:v>
+        <x:v>4fcdcbb818dbd1a28038ad208f7cc0a88cc7fc44e6a708eb8868a7f3f5c6e803</x:v>
       </x:c>
       <x:c r="T199" s="11" t="str">
-        <x:v>d3651428e9d5fb18720ade1cca7a832c2d21a4be2769a1043ead1c2c610bb335</x:v>
+        <x:v>0becf213da9cccd311b61d044d08f29ac420ee2845dd4e9efe9b53c53e822bd3</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="42" customHeight="1">
@@ -15632,7 +15647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1adfb21a56bf4a20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5978b9f9987444d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(v7): deliver v7-4 backend workbook and verified floral handoff
</commit_message>
<xml_diff>
--- a/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
+++ b/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="R1e450220f29c480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="Re3654206f651406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="R9cae78a492644e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="R032d57a7fee34c44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="R003c50fd1d8547c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R509fae8fdbe84437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="R7ca5b101c90c497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="R1ed45773897b4d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="R929891afc87b4b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="R8e7899d0fdef472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="Rf0bd6d5736c54d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R8c557bba695d4a1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,8 +256,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ConfigTable0" displayName="ConfigTable0" ref="A5:H25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:H25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ConfigTable0" displayName="ConfigTable0" ref="A5:H26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:H26"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="字段路径"/>
     <x:tableColumn id="2" name="中文含义"/>
@@ -609,7 +609,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -695,16 +695,16 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
-        <x:v>["v7-1","v7-2","v7-3"]</x:v>
+        <x:v>["v7-1","v7-2","v7-3","v7-4"]</x:v>
       </x:c>
       <x:c r="G7" s="11" t="str">
         <x:v>作品 DesignConfig</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>默认v7-3；旧作品v7-1/v7-2按原版本回放</x:v>
+        <x:v>默认v7-4；旧作品v7-1/v7-2/v7-3按原版本回放</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="55" customHeight="1">
@@ -1125,39 +1125,39 @@
     </x:row>
     <x:row r="24" ht="55" customHeight="1">
       <x:c r="A24" s="10" t="str">
-        <x:v>fixed.atlas</x:v>
+        <x:v>fixedMapping</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>花纸图集分区</x:v>
+        <x:v>固定花纸映射版本</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
-        <x:v>object</x:v>
+        <x:v>string</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
         <x:v>否</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>—</x:v>
+        <x:v>source-layout-v3</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
-        <x:v>随对应资源档位</x:v>
+        <x:v>["source-layout-v3","source-layout-v4"]</x:v>
       </x:c>
       <x:c r="G24" s="10" t="str">
         <x:v>CDN manifest</x:v>
       </x:c>
       <x:c r="H24" s="10" t="str">
-        <x:v>rows/contentWidth/contentHeight/gutter随编译产物保留，不可只换图片尺寸。</x:v>
+        <x:v>v7-4声明source-layout-v4：三部件花纹镜像，杯身花纹底边0.12 mm。缺省按v3。不是DesignConfig字段，不可由后台任意改写旧发布。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="55" customHeight="1">
       <x:c r="A25" s="11" t="str">
-        <x:v>quality / DPR / cache / deviceMemory</x:v>
+        <x:v>fixed.atlas</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>设备与清晰度状态</x:v>
+        <x:v>花纸图集分区</x:v>
       </x:c>
       <x:c r="C25" s="11" t="str">
-        <x:v>runtime</x:v>
+        <x:v>object</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
         <x:v>否</x:v>
@@ -1166,110 +1166,161 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F25" s="11" t="str">
+        <x:v>随对应资源档位</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str">
+        <x:v>CDN manifest</x:v>
+      </x:c>
+      <x:c r="H25" s="11" t="str">
+        <x:v>rows/contentWidth/contentHeight/gutter随编译产物保留，不可只换图片尺寸。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="55" customHeight="1">
+      <x:c r="A26" s="10" t="str">
+        <x:v>quality / DPR / cache / deviceMemory</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>设备与清晰度状态</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>runtime</x:v>
+      </x:c>
+      <x:c r="D26" s="10" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
         <x:v>由前端调度</x:v>
       </x:c>
-      <x:c r="G25" s="11" t="str">
+      <x:c r="G26" s="10" t="str">
         <x:v>不写入作品</x:v>
       </x:c>
-      <x:c r="H25" s="11" t="str">
+      <x:c r="H26" s="10" t="str">
         <x:v>未提供的机器内存指标为不可用；禁止当作0。</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="110" customHeight="1">
-      <x:c r="A28" t="str">
+    <x:row r="29" ht="110" customHeight="1">
+      <x:c r="A29" t="str">
         <x:v>深圳默认作品 JSON（H列完整复制）</x:v>
       </x:c>
-      <x:c r="H28" s="12" t="str">
-        <x:v>{"schemaVersion":1,"resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","cityId":"shenzhen","sloganId":"open","appearance":{"preset":"gold","hue":41.80851063829786,"saturation":100,"lightness":63.13725490196078,"material":1,"materialX":0.5,"relief":1}}</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="34" customHeight="1">
-      <x:c r="A30" t="str">
+      <x:c r="H29" s="12" t="str">
+        <x:v>{"schemaVersion":1,"resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","cityId":"shenzhen","sloganId":"open","appearance":{"preset":"gold","hue":41.80851063829786,"saturation":100,"lightness":63.13725490196078,"material":1,"materialX":0.5,"relief":1}}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="34" customHeight="1">
+      <x:c r="A31" t="str">
         <x:v>数据来源（完整提交与文件哈希见JSON sources）</x:v>
       </x:c>
-      <x:c r="H30" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/package.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="34" customHeight="1">
       <x:c r="H31" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/evidence/v7.1.2/slogans-source.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/package.json</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
       <x:c r="H32" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/evidence/v7.1.2/cities/review.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.3/resource-build.json</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
       <x:c r="H33" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.3/handle-dimensions.json</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
       <x:c r="H34" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/slogans.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/geometry/fixed-mapping.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
       <x:c r="H35" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/style-manager.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
       <x:c r="H36" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/integration/contracts/resource-manifest.schema.json</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="H37" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.2/slogans-source.json</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="H38" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.2/cities/review.json</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="H39" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/types.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="H40" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/design.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/slogans.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
       <x:c r="H41" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="H42" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
       <x:c r="H43" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
       <x:c r="H44" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/releases/v7-3/catalog.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
       <x:c r="H45" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3dee2885886faf4b42f01618593ced0e69b964be/guangcai-china-preview/public/releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/types.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="H46" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/design.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="H47" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="H48" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="H49" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="H50" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/releases/v7-4/catalog.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="H51" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R784db46361f04a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reee7f11b36b347e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1327,7 +1378,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1409,10 +1460,10 @@
         <x:v>上海</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>shanghai-thumbnail</x:v>
@@ -1436,7 +1487,7 @@
         <x:v>shanghai-detail-normal</x:v>
       </x:c>
       <x:c r="M6" s="10" t="str">
-        <x:v>{"cityId":"shanghai","name":"上海","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shanghai-thumbnail","light":{"mask":"shanghai-light-mask","normal":"shanghai-light-normal"},"standard":{"mask":"shanghai-standard-mask","normal":"shanghai-standard-normal"},"detail":{"mask":"shanghai-detail-mask","normal":"shanghai-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shanghai","name":"上海","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"shanghai-thumbnail","light":{"mask":"shanghai-light-mask","normal":"shanghai-light-normal"},"standard":{"mask":"shanghai-standard-mask","normal":"shanghai-standard-normal"},"detail":{"mask":"shanghai-detail-mask","normal":"shanghai-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
@@ -1450,10 +1501,10 @@
         <x:v>乌鲁木齐</x:v>
       </x:c>
       <x:c r="D7" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F7" s="11" t="str">
         <x:v>urumqi-thumbnail</x:v>
@@ -1477,7 +1528,7 @@
         <x:v>urumqi-detail-normal</x:v>
       </x:c>
       <x:c r="M7" s="11" t="str">
-        <x:v>{"cityId":"urumqi","name":"乌鲁木齐","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"urumqi-thumbnail","light":{"mask":"urumqi-light-mask","normal":"urumqi-light-normal"},"standard":{"mask":"urumqi-standard-mask","normal":"urumqi-standard-normal"},"detail":{"mask":"urumqi-detail-mask","normal":"urumqi-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"urumqi","name":"乌鲁木齐","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"urumqi-thumbnail","light":{"mask":"urumqi-light-mask","normal":"urumqi-light-normal"},"standard":{"mask":"urumqi-standard-mask","normal":"urumqi-standard-normal"},"detail":{"mask":"urumqi-detail-mask","normal":"urumqi-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
@@ -1491,10 +1542,10 @@
         <x:v>北京</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>beijing-thumbnail</x:v>
@@ -1518,7 +1569,7 @@
         <x:v>beijing-detail-normal</x:v>
       </x:c>
       <x:c r="M8" s="10" t="str">
-        <x:v>{"cityId":"beijing","name":"北京","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"beijing-thumbnail","light":{"mask":"beijing-light-mask","normal":"beijing-light-normal"},"standard":{"mask":"beijing-standard-mask","normal":"beijing-standard-normal"},"detail":{"mask":"beijing-detail-mask","normal":"beijing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"beijing","name":"北京","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"beijing-thumbnail","light":{"mask":"beijing-light-mask","normal":"beijing-light-normal"},"standard":{"mask":"beijing-standard-mask","normal":"beijing-standard-normal"},"detail":{"mask":"beijing-detail-mask","normal":"beijing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
@@ -1532,10 +1583,10 @@
         <x:v>南京</x:v>
       </x:c>
       <x:c r="D9" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
         <x:v>nanjing-thumbnail</x:v>
@@ -1559,7 +1610,7 @@
         <x:v>nanjing-detail-normal</x:v>
       </x:c>
       <x:c r="M9" s="11" t="str">
-        <x:v>{"cityId":"nanjing","name":"南京","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"nanjing-thumbnail","light":{"mask":"nanjing-light-mask","normal":"nanjing-light-normal"},"standard":{"mask":"nanjing-standard-mask","normal":"nanjing-standard-normal"},"detail":{"mask":"nanjing-detail-mask","normal":"nanjing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"nanjing","name":"南京","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"nanjing-thumbnail","light":{"mask":"nanjing-light-mask","normal":"nanjing-light-normal"},"standard":{"mask":"nanjing-standard-mask","normal":"nanjing-standard-normal"},"detail":{"mask":"nanjing-detail-mask","normal":"nanjing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
@@ -1573,10 +1624,10 @@
         <x:v>南昌</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
         <x:v>nanchang-thumbnail</x:v>
@@ -1600,7 +1651,7 @@
         <x:v>nanchang-detail-normal</x:v>
       </x:c>
       <x:c r="M10" s="10" t="str">
-        <x:v>{"cityId":"nanchang","name":"南昌","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"nanchang-thumbnail","light":{"mask":"nanchang-light-mask","normal":"nanchang-light-normal"},"standard":{"mask":"nanchang-standard-mask","normal":"nanchang-standard-normal"},"detail":{"mask":"nanchang-detail-mask","normal":"nanchang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"nanchang","name":"南昌","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"nanchang-thumbnail","light":{"mask":"nanchang-light-mask","normal":"nanchang-light-normal"},"standard":{"mask":"nanchang-standard-mask","normal":"nanchang-standard-normal"},"detail":{"mask":"nanchang-detail-mask","normal":"nanchang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
@@ -1614,10 +1665,10 @@
         <x:v>厦门</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
         <x:v>xiamen-thumbnail</x:v>
@@ -1641,7 +1692,7 @@
         <x:v>xiamen-detail-normal</x:v>
       </x:c>
       <x:c r="M11" s="11" t="str">
-        <x:v>{"cityId":"xiamen","name":"厦门","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"xiamen-thumbnail","light":{"mask":"xiamen-light-mask","normal":"xiamen-light-normal"},"standard":{"mask":"xiamen-standard-mask","normal":"xiamen-standard-normal"},"detail":{"mask":"xiamen-detail-mask","normal":"xiamen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"xiamen","name":"厦门","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"xiamen-thumbnail","light":{"mask":"xiamen-light-mask","normal":"xiamen-light-normal"},"standard":{"mask":"xiamen-standard-mask","normal":"xiamen-standard-normal"},"detail":{"mask":"xiamen-detail-mask","normal":"xiamen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
@@ -1655,10 +1706,10 @@
         <x:v>呼和浩特</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
         <x:v>hohhot-thumbnail</x:v>
@@ -1682,7 +1733,7 @@
         <x:v>hohhot-detail-normal</x:v>
       </x:c>
       <x:c r="M12" s="10" t="str">
-        <x:v>{"cityId":"hohhot","name":"呼和浩特","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"hohhot-thumbnail","light":{"mask":"hohhot-light-mask","normal":"hohhot-light-normal"},"standard":{"mask":"hohhot-standard-mask","normal":"hohhot-standard-normal"},"detail":{"mask":"hohhot-detail-mask","normal":"hohhot-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"hohhot","name":"呼和浩特","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"hohhot-thumbnail","light":{"mask":"hohhot-light-mask","normal":"hohhot-light-normal"},"standard":{"mask":"hohhot-standard-mask","normal":"hohhot-standard-normal"},"detail":{"mask":"hohhot-detail-mask","normal":"hohhot-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
@@ -1696,10 +1747,10 @@
         <x:v>哈尔滨</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
         <x:v>harbin-thumbnail</x:v>
@@ -1723,7 +1774,7 @@
         <x:v>harbin-detail-normal</x:v>
       </x:c>
       <x:c r="M13" s="11" t="str">
-        <x:v>{"cityId":"harbin","name":"哈尔滨","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"harbin-thumbnail","light":{"mask":"harbin-light-mask","normal":"harbin-light-normal"},"standard":{"mask":"harbin-standard-mask","normal":"harbin-standard-normal"},"detail":{"mask":"harbin-detail-mask","normal":"harbin-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"harbin","name":"哈尔滨","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"harbin-thumbnail","light":{"mask":"harbin-light-mask","normal":"harbin-light-normal"},"standard":{"mask":"harbin-standard-mask","normal":"harbin-standard-normal"},"detail":{"mask":"harbin-detail-mask","normal":"harbin-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1737,10 +1788,10 @@
         <x:v>天津</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>tianjin-thumbnail</x:v>
@@ -1764,7 +1815,7 @@
         <x:v>tianjin-detail-normal</x:v>
       </x:c>
       <x:c r="M14" s="10" t="str">
-        <x:v>{"cityId":"tianjin","name":"天津","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"tianjin-thumbnail","light":{"mask":"tianjin-light-mask","normal":"tianjin-light-normal"},"standard":{"mask":"tianjin-standard-mask","normal":"tianjin-standard-normal"},"detail":{"mask":"tianjin-detail-mask","normal":"tianjin-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"tianjin","name":"天津","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"tianjin-thumbnail","light":{"mask":"tianjin-light-mask","normal":"tianjin-light-normal"},"standard":{"mask":"tianjin-standard-mask","normal":"tianjin-standard-normal"},"detail":{"mask":"tianjin-detail-mask","normal":"tianjin-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
@@ -1778,10 +1829,10 @@
         <x:v>太原</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
         <x:v>taiyuan-thumbnail</x:v>
@@ -1805,7 +1856,7 @@
         <x:v>taiyuan-detail-normal</x:v>
       </x:c>
       <x:c r="M15" s="11" t="str">
-        <x:v>{"cityId":"taiyuan","name":"太原","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"taiyuan-thumbnail","light":{"mask":"taiyuan-light-mask","normal":"taiyuan-light-normal"},"standard":{"mask":"taiyuan-standard-mask","normal":"taiyuan-standard-normal"},"detail":{"mask":"taiyuan-detail-mask","normal":"taiyuan-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"taiyuan","name":"太原","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"taiyuan-thumbnail","light":{"mask":"taiyuan-light-mask","normal":"taiyuan-light-normal"},"standard":{"mask":"taiyuan-standard-mask","normal":"taiyuan-standard-normal"},"detail":{"mask":"taiyuan-detail-mask","normal":"taiyuan-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
@@ -1819,10 +1870,10 @@
         <x:v>广州</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
         <x:v>guangzhou-thumbnail</x:v>
@@ -1846,7 +1897,7 @@
         <x:v>guangzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M16" s="10" t="str">
-        <x:v>{"cityId":"guangzhou","name":"广州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"guangzhou-thumbnail","light":{"mask":"guangzhou-light-mask","normal":"guangzhou-light-normal"},"standard":{"mask":"guangzhou-standard-mask","normal":"guangzhou-standard-normal"},"detail":{"mask":"guangzhou-detail-mask","normal":"guangzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"guangzhou","name":"广州","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"guangzhou-thumbnail","light":{"mask":"guangzhou-light-mask","normal":"guangzhou-light-normal"},"standard":{"mask":"guangzhou-standard-mask","normal":"guangzhou-standard-normal"},"detail":{"mask":"guangzhou-detail-mask","normal":"guangzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
@@ -1860,10 +1911,10 @@
         <x:v>成都</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E17" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
         <x:v>chengdu-thumbnail</x:v>
@@ -1887,7 +1938,7 @@
         <x:v>chengdu-detail-normal</x:v>
       </x:c>
       <x:c r="M17" s="11" t="str">
-        <x:v>{"cityId":"chengdu","name":"成都","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"chengdu-thumbnail","light":{"mask":"chengdu-light-mask","normal":"chengdu-light-normal"},"standard":{"mask":"chengdu-standard-mask","normal":"chengdu-standard-normal"},"detail":{"mask":"chengdu-detail-mask","normal":"chengdu-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"chengdu","name":"成都","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"chengdu-thumbnail","light":{"mask":"chengdu-light-mask","normal":"chengdu-light-normal"},"standard":{"mask":"chengdu-standard-mask","normal":"chengdu-standard-normal"},"detail":{"mask":"chengdu-detail-mask","normal":"chengdu-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -1901,10 +1952,10 @@
         <x:v>景德镇</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E18" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F18" s="10" t="str">
         <x:v>jingdezhen-thumbnail</x:v>
@@ -1928,7 +1979,7 @@
         <x:v>jingdezhen-detail-normal</x:v>
       </x:c>
       <x:c r="M18" s="10" t="str">
-        <x:v>{"cityId":"jingdezhen","name":"景德镇","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"jingdezhen-thumbnail","light":{"mask":"jingdezhen-light-mask","normal":"jingdezhen-light-normal"},"standard":{"mask":"jingdezhen-standard-mask","normal":"jingdezhen-standard-normal"},"detail":{"mask":"jingdezhen-detail-mask","normal":"jingdezhen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"jingdezhen","name":"景德镇","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"jingdezhen-thumbnail","light":{"mask":"jingdezhen-light-mask","normal":"jingdezhen-light-normal"},"standard":{"mask":"jingdezhen-standard-mask","normal":"jingdezhen-standard-normal"},"detail":{"mask":"jingdezhen-detail-mask","normal":"jingdezhen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -1942,10 +1993,10 @@
         <x:v>杭州</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E19" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F19" s="11" t="str">
         <x:v>hangzhou-thumbnail</x:v>
@@ -1969,7 +2020,7 @@
         <x:v>hangzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M19" s="11" t="str">
-        <x:v>{"cityId":"hangzhou","name":"杭州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"hangzhou-thumbnail","light":{"mask":"hangzhou-light-mask","normal":"hangzhou-light-normal"},"standard":{"mask":"hangzhou-standard-mask","normal":"hangzhou-standard-normal"},"detail":{"mask":"hangzhou-detail-mask","normal":"hangzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"hangzhou","name":"杭州","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"hangzhou-thumbnail","light":{"mask":"hangzhou-light-mask","normal":"hangzhou-light-normal"},"standard":{"mask":"hangzhou-standard-mask","normal":"hangzhou-standard-normal"},"detail":{"mask":"hangzhou-detail-mask","normal":"hangzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -1983,10 +2034,10 @@
         <x:v>武汉</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E20" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F20" s="10" t="str">
         <x:v>wuhan-thumbnail</x:v>
@@ -2010,7 +2061,7 @@
         <x:v>wuhan-detail-normal</x:v>
       </x:c>
       <x:c r="M20" s="10" t="str">
-        <x:v>{"cityId":"wuhan","name":"武汉","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"wuhan-thumbnail","light":{"mask":"wuhan-light-mask","normal":"wuhan-light-normal"},"standard":{"mask":"wuhan-standard-mask","normal":"wuhan-standard-normal"},"detail":{"mask":"wuhan-detail-mask","normal":"wuhan-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"wuhan","name":"武汉","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"wuhan-thumbnail","light":{"mask":"wuhan-light-mask","normal":"wuhan-light-normal"},"standard":{"mask":"wuhan-standard-mask","normal":"wuhan-standard-normal"},"detail":{"mask":"wuhan-detail-mask","normal":"wuhan-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -2024,10 +2075,10 @@
         <x:v>沈阳</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
         <x:v>shenyang-thumbnail</x:v>
@@ -2051,7 +2102,7 @@
         <x:v>shenyang-detail-normal</x:v>
       </x:c>
       <x:c r="M21" s="11" t="str">
-        <x:v>{"cityId":"shenyang","name":"沈阳","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shenyang-thumbnail","light":{"mask":"shenyang-light-mask","normal":"shenyang-light-normal"},"standard":{"mask":"shenyang-standard-mask","normal":"shenyang-standard-normal"},"detail":{"mask":"shenyang-detail-mask","normal":"shenyang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shenyang","name":"沈阳","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"shenyang-thumbnail","light":{"mask":"shenyang-light-mask","normal":"shenyang-light-normal"},"standard":{"mask":"shenyang-standard-mask","normal":"shenyang-standard-normal"},"detail":{"mask":"shenyang-detail-mask","normal":"shenyang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -2065,10 +2116,10 @@
         <x:v>深圳</x:v>
       </x:c>
       <x:c r="D22" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E22" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F22" s="10" t="str">
         <x:v>shenzhen-thumbnail</x:v>
@@ -2092,7 +2143,7 @@
         <x:v>shenzhen-detail-normal</x:v>
       </x:c>
       <x:c r="M22" s="10" t="str">
-        <x:v>{"cityId":"shenzhen","name":"深圳","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shenzhen-thumbnail","light":{"mask":"shenzhen-light-mask","normal":"shenzhen-light-normal"},"standard":{"mask":"shenzhen-standard-mask","normal":"shenzhen-standard-normal"},"detail":{"mask":"shenzhen-detail-mask","normal":"shenzhen-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shenzhen","name":"深圳","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"shenzhen-thumbnail","light":{"mask":"shenzhen-light-mask","normal":"shenzhen-light-normal"},"standard":{"mask":"shenzhen-standard-mask","normal":"shenzhen-standard-normal"},"detail":{"mask":"shenzhen-detail-mask","normal":"shenzhen-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -2106,10 +2157,10 @@
         <x:v>石家庄</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E23" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F23" s="11" t="str">
         <x:v>shijiazhuang-thumbnail</x:v>
@@ -2133,7 +2184,7 @@
         <x:v>shijiazhuang-detail-normal</x:v>
       </x:c>
       <x:c r="M23" s="11" t="str">
-        <x:v>{"cityId":"shijiazhuang","name":"石家庄","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"shijiazhuang-thumbnail","light":{"mask":"shijiazhuang-light-mask","normal":"shijiazhuang-light-normal"},"standard":{"mask":"shijiazhuang-standard-mask","normal":"shijiazhuang-standard-normal"},"detail":{"mask":"shijiazhuang-detail-mask","normal":"shijiazhuang-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"shijiazhuang","name":"石家庄","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"shijiazhuang-thumbnail","light":{"mask":"shijiazhuang-light-mask","normal":"shijiazhuang-light-normal"},"standard":{"mask":"shijiazhuang-standard-mask","normal":"shijiazhuang-standard-normal"},"detail":{"mask":"shijiazhuang-detail-mask","normal":"shijiazhuang-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
@@ -2147,10 +2198,10 @@
         <x:v>西安</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
         <x:v>xian-thumbnail</x:v>
@@ -2174,7 +2225,7 @@
         <x:v>xian-detail-normal</x:v>
       </x:c>
       <x:c r="M24" s="10" t="str">
-        <x:v>{"cityId":"xian","name":"西安","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"xian-thumbnail","light":{"mask":"xian-light-mask","normal":"xian-light-normal"},"standard":{"mask":"xian-standard-mask","normal":"xian-standard-normal"},"detail":{"mask":"xian-detail-mask","normal":"xian-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"xian","name":"西安","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"xian-thumbnail","light":{"mask":"xian-light-mask","normal":"xian-light-normal"},"standard":{"mask":"xian-standard-mask","normal":"xian-standard-normal"},"detail":{"mask":"xian-detail-mask","normal":"xian-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
@@ -2188,10 +2239,10 @@
         <x:v>郑州</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E25" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F25" s="11" t="str">
         <x:v>zhengzhou-thumbnail</x:v>
@@ -2215,7 +2266,7 @@
         <x:v>zhengzhou-detail-normal</x:v>
       </x:c>
       <x:c r="M25" s="11" t="str">
-        <x:v>{"cityId":"zhengzhou","name":"郑州","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"zhengzhou-thumbnail","light":{"mask":"zhengzhou-light-mask","normal":"zhengzhou-light-normal"},"standard":{"mask":"zhengzhou-standard-mask","normal":"zhengzhou-standard-normal"},"detail":{"mask":"zhengzhou-detail-mask","normal":"zhengzhou-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"zhengzhou","name":"郑州","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"zhengzhou-thumbnail","light":{"mask":"zhengzhou-light-mask","normal":"zhengzhou-light-normal"},"standard":{"mask":"zhengzhou-standard-mask","normal":"zhengzhou-standard-normal"},"detail":{"mask":"zhengzhou-detail-mask","normal":"zhengzhou-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
@@ -2229,10 +2280,10 @@
         <x:v>重庆</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F26" s="10" t="str">
         <x:v>chongqing-thumbnail</x:v>
@@ -2256,7 +2307,7 @@
         <x:v>chongqing-detail-normal</x:v>
       </x:c>
       <x:c r="M26" s="10" t="str">
-        <x:v>{"cityId":"chongqing","name":"重庆","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"chongqing-thumbnail","light":{"mask":"chongqing-light-mask","normal":"chongqing-light-normal"},"standard":{"mask":"chongqing-standard-mask","normal":"chongqing-standard-normal"},"detail":{"mask":"chongqing-detail-mask","normal":"chongqing-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"chongqing","name":"重庆","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"chongqing-thumbnail","light":{"mask":"chongqing-light-mask","normal":"chongqing-light-normal"},"standard":{"mask":"chongqing-standard-mask","normal":"chongqing-standard-normal"},"detail":{"mask":"chongqing-detail-mask","normal":"chongqing-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -2270,10 +2321,10 @@
         <x:v>长春</x:v>
       </x:c>
       <x:c r="D27" s="11" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E27" s="11" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F27" s="11" t="str">
         <x:v>changchun-thumbnail</x:v>
@@ -2297,7 +2348,7 @@
         <x:v>changchun-detail-normal</x:v>
       </x:c>
       <x:c r="M27" s="11" t="str">
-        <x:v>{"cityId":"changchun","name":"长春","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"changchun-thumbnail","light":{"mask":"changchun-light-mask","normal":"changchun-light-normal"},"standard":{"mask":"changchun-standard-mask","normal":"changchun-standard-normal"},"detail":{"mask":"changchun-detail-mask","normal":"changchun-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"changchun","name":"长春","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"changchun-thumbnail","light":{"mask":"changchun-light-mask","normal":"changchun-light-normal"},"standard":{"mask":"changchun-standard-mask","normal":"changchun-standard-normal"},"detail":{"mask":"changchun-detail-mask","normal":"changchun-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -2311,10 +2362,10 @@
         <x:v>青岛</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>v7-3</x:v>
+        <x:v>v7-4</x:v>
       </x:c>
       <x:c r="E28" s="10" t="str">
-        <x:v>releases/v7-3/manifest-b27eb343b846cdc4.json</x:v>
+        <x:v>releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
       <x:c r="F28" s="10" t="str">
         <x:v>qingdao-thumbnail</x:v>
@@ -2338,13 +2389,13 @@
         <x:v>qingdao-detail-normal</x:v>
       </x:c>
       <x:c r="M28" s="10" t="str">
-        <x:v>{"cityId":"qingdao","name":"青岛","resourceReleaseId":"v7-3","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-3/manifest-b27eb343b846cdc4.json","resourceIds":{"thumbnail":"qingdao-thumbnail","light":{"mask":"qingdao-light-mask","normal":"qingdao-light-normal"},"standard":{"mask":"qingdao-standard-mask","normal":"qingdao-standard-normal"},"detail":{"mask":"qingdao-detail-mask","normal":"qingdao-detail-normal"}}}</x:v>
+        <x:v>{"cityId":"qingdao","name":"青岛","resourceReleaseId":"v7-4","modelVersion":"china-cup-v6","recipeVersion":"porcelain-city-v6","manifestUrl":"releases/v7-4/manifest-a6484ca5de3f4cc2.json","resourceIds":{"thumbnail":"qingdao-thumbnail","light":{"mask":"qingdao-light-mask","normal":"qingdao-light-normal"},"standard":{"mask":"qingdao-standard-mask","normal":"qingdao-standard-normal"},"detail":{"mask":"qingdao-detail-mask","normal":"qingdao-detail-normal"}}}</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73ce3e95983e4d98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6a45a59bf5c4e10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2405,7 +2456,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2714,7 +2765,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2333119161614b6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde0c29b00504b0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2757,7 +2808,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3121,7 +3172,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4989efc715743a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c8aa1c35ee140dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3164,7 +3215,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3233,7 +3284,7 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H6" s="10" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="65" customHeight="1">
@@ -3259,7 +3310,7 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H7" s="11" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="65" customHeight="1">
@@ -3285,7 +3336,7 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65" customHeight="1">
@@ -3311,7 +3362,7 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="65" customHeight="1">
@@ -3337,7 +3388,7 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="65" customHeight="1">
@@ -3363,13 +3414,13 @@
         <x:v>[0.77490234375,0.38754907459338195,0.0703125,0.5249579360628155]</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>Source Han Serif CN Bold 700；v7-3；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
+        <x:v>Source Han Serif CN Bold 700；v7-4；WebP线性R8；4px护边；六组首屏预热；字体仅制作使用</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ed795bf71f94bf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf7fc22a5fa146ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3448,7 +3499,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.2 / v7-3 / 3dee2885886f · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3583,7 +3634,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J6" s="14" t="n">
-        <x:v>151206</x:v>
+        <x:v>149578</x:v>
       </x:c>
       <x:c r="K6" s="14" t="n">
         <x:v>1740800</x:v>
@@ -3601,19 +3652,19 @@
         <x:v>2321067</x:v>
       </x:c>
       <x:c r="P6" s="10" t="str">
-        <x:v>../v7-1/assets/fixed-body-light-color-8c2bf9cbe44a3d18.webp</x:v>
+        <x:v>assets/fixed-body-light-color-f4e419cd29c55ac9.webp</x:v>
       </x:c>
       <x:c r="Q6" s="10" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-light-color-8c2bf9cbe44a3d18.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-light-color-f4e419cd29c55ac9.webp</x:v>
       </x:c>
       <x:c r="R6" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-light-color-8c2bf9cbe44a3d18.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-light-color-f4e419cd29c55ac9.webp</x:v>
       </x:c>
       <x:c r="S6" s="10" t="str">
-        <x:v>8c2bf9cbe44a3d18658ede38822ce091abbcd9cfb3dbcf07557edede50cb97e7</x:v>
+        <x:v>f4e419cd29c55ac986eecd36759d988e8c72a9c2c56ba9c37176008f1de0b0d4</x:v>
       </x:c>
       <x:c r="T6" s="10" t="str">
-        <x:v>973cf1048f697acafd3bbe3f4bbdf6eb9ba46469572e571e35c1c5fad12d6559</x:v>
+        <x:v>ccb2af98157bccbf9ae97358371669fa0a3488ce709f926e1cb451c28809282e</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -3645,7 +3696,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J7" s="16" t="n">
-        <x:v>915743</x:v>
+        <x:v>910683</x:v>
       </x:c>
       <x:c r="K7" s="16" t="n">
         <x:v>3481600</x:v>
@@ -3663,19 +3714,19 @@
         <x:v>2321067</x:v>
       </x:c>
       <x:c r="P7" s="11" t="str">
-        <x:v>../v7-1/assets/fixed-body-light-normal-fc1a43461e425077.hfn.gz</x:v>
+        <x:v>assets/fixed-body-light-normal-21b9894d6ea0354a.hfn.gz</x:v>
       </x:c>
       <x:c r="Q7" s="11" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-light-normal-fc1a43461e425077.hfn.gz</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-light-normal-21b9894d6ea0354a.hfn.gz</x:v>
       </x:c>
       <x:c r="R7" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-light-normal-fc1a43461e425077.hfn.gz</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-light-normal-21b9894d6ea0354a.hfn.gz</x:v>
       </x:c>
       <x:c r="S7" s="11" t="str">
-        <x:v>fc1a43461e4250778580bc90584a118e7ce2a694864bf5d10fa539887fa6058d</x:v>
+        <x:v>21b9894d6ea0354a43660e3e00d8b4c5b49212b814d3d665415631e2076e02b9</x:v>
       </x:c>
       <x:c r="T7" s="11" t="str">
-        <x:v>35f734f1f0e183864ac76dd6d7866f7e8c7eadf17f9e287950a986abb943b3db</x:v>
+        <x:v>49b67ebbd362810945e5f62812cd2b18b6de7838e3e86f9cf51149ebe1c6c5c9</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -3707,7 +3758,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J8" s="14" t="n">
-        <x:v>113944</x:v>
+        <x:v>112240</x:v>
       </x:c>
       <x:c r="K8" s="14" t="n">
         <x:v>1740800</x:v>
@@ -3725,19 +3776,19 @@
         <x:v>2321067</x:v>
       </x:c>
       <x:c r="P8" s="10" t="str">
-        <x:v>../v7-1/assets/fixed-body-light-orm-038b21ee36c53021.webp</x:v>
+        <x:v>assets/fixed-body-light-orm-489ca56853301382.webp</x:v>
       </x:c>
       <x:c r="Q8" s="10" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-light-orm-038b21ee36c53021.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-light-orm-489ca56853301382.webp</x:v>
       </x:c>
       <x:c r="R8" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-light-orm-038b21ee36c53021.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-light-orm-489ca56853301382.webp</x:v>
       </x:c>
       <x:c r="S8" s="10" t="str">
-        <x:v>038b21ee36c530210af1767d212b5fae5a293adeffbb19dd2c94046e7a89bbe2</x:v>
+        <x:v>489ca56853301382445e8ac9ad23676c673c1af4cc910f890d5e15d7143e6904</x:v>
       </x:c>
       <x:c r="T8" s="10" t="str">
-        <x:v>f131df6c732aa03d2f7fd0b13cdf9912926a9410f96370f4417ee6c376f5b768</x:v>
+        <x:v>621f23235db6c40f363595c364336a78e070a17eed0578d883e385f1211845db</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -3769,7 +3820,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J9" s="16" t="n">
-        <x:v>389520</x:v>
+        <x:v>386446</x:v>
       </x:c>
       <x:c r="K9" s="16" t="n">
         <x:v>6963200</x:v>
@@ -3787,19 +3838,19 @@
         <x:v>9284267</x:v>
       </x:c>
       <x:c r="P9" s="11" t="str">
-        <x:v>../v7-1/assets/fixed-body-standard-color-6f9be4cd52c23e29.webp</x:v>
+        <x:v>assets/fixed-body-standard-color-bb91f401684f96e5.webp</x:v>
       </x:c>
       <x:c r="Q9" s="11" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-standard-color-6f9be4cd52c23e29.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-standard-color-bb91f401684f96e5.webp</x:v>
       </x:c>
       <x:c r="R9" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-standard-color-6f9be4cd52c23e29.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-standard-color-bb91f401684f96e5.webp</x:v>
       </x:c>
       <x:c r="S9" s="11" t="str">
-        <x:v>6f9be4cd52c23e293a2f608eabb4106b22fdabf46f7583ade448798e662ccdc0</x:v>
+        <x:v>bb91f401684f96e5ae97c594241843b168457781aa121e7121f381fcef704474</x:v>
       </x:c>
       <x:c r="T9" s="11" t="str">
-        <x:v>973cf1048f697acafd3bbe3f4bbdf6eb9ba46469572e571e35c1c5fad12d6559</x:v>
+        <x:v>ccb2af98157bccbf9ae97358371669fa0a3488ce709f926e1cb451c28809282e</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -3831,7 +3882,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J10" s="14" t="n">
-        <x:v>3466614</x:v>
+        <x:v>3449729</x:v>
       </x:c>
       <x:c r="K10" s="14" t="n">
         <x:v>13926400</x:v>
@@ -3849,19 +3900,19 @@
         <x:v>9284267</x:v>
       </x:c>
       <x:c r="P10" s="10" t="str">
-        <x:v>../v7-1/assets/fixed-body-standard-normal-433099d227c03917.hfn.gz</x:v>
+        <x:v>assets/fixed-body-standard-normal-f4b16839dd597ac4.hfn.gz</x:v>
       </x:c>
       <x:c r="Q10" s="10" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-standard-normal-433099d227c03917.hfn.gz</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-standard-normal-f4b16839dd597ac4.hfn.gz</x:v>
       </x:c>
       <x:c r="R10" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-standard-normal-433099d227c03917.hfn.gz</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-standard-normal-f4b16839dd597ac4.hfn.gz</x:v>
       </x:c>
       <x:c r="S10" s="10" t="str">
-        <x:v>433099d227c039173c918048bfdf3c3d4b9056d12eb864ad795e8c56891d7022</x:v>
+        <x:v>f4b16839dd597ac489b0ddfb52e10da9dfdd1957b0c7ee502a86142a9060af06</x:v>
       </x:c>
       <x:c r="T10" s="10" t="str">
-        <x:v>35f734f1f0e183864ac76dd6d7866f7e8c7eadf17f9e287950a986abb943b3db</x:v>
+        <x:v>49b67ebbd362810945e5f62812cd2b18b6de7838e3e86f9cf51149ebe1c6c5c9</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -3893,7 +3944,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J11" s="16" t="n">
-        <x:v>284336</x:v>
+        <x:v>281146</x:v>
       </x:c>
       <x:c r="K11" s="16" t="n">
         <x:v>6963200</x:v>
@@ -3911,19 +3962,19 @@
         <x:v>9284267</x:v>
       </x:c>
       <x:c r="P11" s="11" t="str">
-        <x:v>../v7-1/assets/fixed-body-standard-orm-4738736a95e92256.webp</x:v>
+        <x:v>assets/fixed-body-standard-orm-4be928717d848cca.webp</x:v>
       </x:c>
       <x:c r="Q11" s="11" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-standard-orm-4738736a95e92256.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-standard-orm-4be928717d848cca.webp</x:v>
       </x:c>
       <x:c r="R11" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-standard-orm-4738736a95e92256.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-standard-orm-4be928717d848cca.webp</x:v>
       </x:c>
       <x:c r="S11" s="11" t="str">
-        <x:v>4738736a95e92256e14a8e98e08ecc9a47cabefe79c154082ac221db3b0aa629</x:v>
+        <x:v>4be928717d848cca46280c286ab73107461957527c8c27e7172271656b28cb5f</x:v>
       </x:c>
       <x:c r="T11" s="11" t="str">
-        <x:v>f131df6c732aa03d2f7fd0b13cdf9912926a9410f96370f4417ee6c376f5b768</x:v>
+        <x:v>621f23235db6c40f363595c364336a78e070a17eed0578d883e385f1211845db</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -3955,7 +4006,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J12" s="14" t="n">
-        <x:v>479504</x:v>
+        <x:v>475446</x:v>
       </x:c>
       <x:c r="K12" s="14" t="n">
         <x:v>10100736</x:v>
@@ -3973,19 +4024,19 @@
         <x:v>13467648</x:v>
       </x:c>
       <x:c r="P12" s="10" t="str">
-        <x:v>../v7-1/assets/fixed-body-detail-color-667b175ba4181dce.webp</x:v>
+        <x:v>assets/fixed-body-detail-color-55458633cf881236.webp</x:v>
       </x:c>
       <x:c r="Q12" s="10" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-detail-color-667b175ba4181dce.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-detail-color-55458633cf881236.webp</x:v>
       </x:c>
       <x:c r="R12" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-detail-color-667b175ba4181dce.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-detail-color-55458633cf881236.webp</x:v>
       </x:c>
       <x:c r="S12" s="10" t="str">
-        <x:v>667b175ba4181dce310c7214424116909e0d2fa60aa63ac1c78bf6d63da1edd1</x:v>
+        <x:v>55458633cf881236e5bc51fce2aaffcde06cc08e4e438b245392eac2ae7b3245</x:v>
       </x:c>
       <x:c r="T12" s="10" t="str">
-        <x:v>973cf1048f697acafd3bbe3f4bbdf6eb9ba46469572e571e35c1c5fad12d6559</x:v>
+        <x:v>ccb2af98157bccbf9ae97358371669fa0a3488ce709f926e1cb451c28809282e</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -4017,7 +4068,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J13" s="16" t="n">
-        <x:v>4959453</x:v>
+        <x:v>4845924</x:v>
       </x:c>
       <x:c r="K13" s="16" t="n">
         <x:v>20201472</x:v>
@@ -4035,19 +4086,19 @@
         <x:v>13467648</x:v>
       </x:c>
       <x:c r="P13" s="11" t="str">
-        <x:v>../v7-1/assets/fixed-body-detail-normal-35f734f1f0e18386.hfn.gz</x:v>
+        <x:v>assets/fixed-body-detail-normal-49b67ebbd3628109.hfn.gz</x:v>
       </x:c>
       <x:c r="Q13" s="11" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-detail-normal-35f734f1f0e18386.hfn.gz</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-detail-normal-49b67ebbd3628109.hfn.gz</x:v>
       </x:c>
       <x:c r="R13" s="11" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-detail-normal-35f734f1f0e18386.hfn.gz</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-detail-normal-49b67ebbd3628109.hfn.gz</x:v>
       </x:c>
       <x:c r="S13" s="11" t="str">
-        <x:v>35f734f1f0e183864ac76dd6d7866f7e8c7eadf17f9e287950a986abb943b3db</x:v>
+        <x:v>49b67ebbd362810945e5f62812cd2b18b6de7838e3e86f9cf51149ebe1c6c5c9</x:v>
       </x:c>
       <x:c r="T13" s="11" t="str">
-        <x:v>35f734f1f0e183864ac76dd6d7866f7e8c7eadf17f9e287950a986abb943b3db</x:v>
+        <x:v>49b67ebbd362810945e5f62812cd2b18b6de7838e3e86f9cf51149ebe1c6c5c9</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -4079,7 +4130,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="J14" s="14" t="n">
-        <x:v>282582</x:v>
+        <x:v>281864</x:v>
       </x:c>
       <x:c r="K14" s="14" t="n">
         <x:v>10100736</x:v>
@@ -4097,19 +4148,19 @@
         <x:v>13467648</x:v>
       </x:c>
       <x:c r="P14" s="10" t="str">
-        <x:v>../v7-1/assets/fixed-body-detail-orm-2f29c84c7465fc11.webp</x:v>
+        <x:v>assets/fixed-body-detail-orm-a117af74f734bf7d.webp</x:v>
       </x:c>
       <x:c r="Q14" s="10" t="str">
-        <x:v>releases/v7-1/assets/fixed-body-detail-orm-2f29c84c7465fc11.webp</x:v>
+        <x:v>releases/v7-4/assets/fixed-body-detail-orm-a117af74f734bf7d.webp</x:v>
       </x:c>
       <x:c r="R14" s="10" t="str">
-        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-1/assets/fixed-body-detail-orm-2f29c84c7465fc11.webp</x:v>
+        <x:v>https://guangcai-no1-china-v7.netlify.app/releases/v7-4/assets/fixed-body-detail-orm-a117af74f734bf7d.webp</x:v>
       </x:c>
       <x:c r="S14" s="10" t="str">
-        <x:v>2f29c84c7465fc11947162789e344dd257faf56c173546c8d47056e341b54681</x:v>
+        <x:v>a117af74f734bf7d1b175ca4b31c5e0ad40244b49a78d32ed1ff5bd538685e4b</x:v>
       </x:c>
       <x:c r="T14" s="10" t="str">
-        <x:v>f131df6c732aa03d2f7fd0b13cdf9912926a9410f96370f4417ee6c376f5b768</x:v>
+        <x:v>621f23235db6c40f363595c364336a78e070a17eed0578d883e385f1211845db</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -7507,7 +7558,7 @@
         <x:v>1217878</x:v>
       </x:c>
       <x:c r="P69" s="11" t="str">
-        <x:v>assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
+        <x:v>../v7-3/assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
       </x:c>
       <x:c r="Q69" s="11" t="str">
         <x:v>releases/v7-3/assets/xiamen-light-mask-43538debb37bd826.webp</x:v>
@@ -7631,7 +7682,7 @@
         <x:v>4871510</x:v>
       </x:c>
       <x:c r="P71" s="11" t="str">
-        <x:v>assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
+        <x:v>../v7-3/assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
       </x:c>
       <x:c r="Q71" s="11" t="str">
         <x:v>releases/v7-3/assets/xiamen-standard-mask-403c47be25586d7a.webp</x:v>
@@ -7755,7 +7806,7 @@
         <x:v>19475115</x:v>
       </x:c>
       <x:c r="P73" s="11" t="str">
-        <x:v>assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
+        <x:v>../v7-3/assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
       </x:c>
       <x:c r="Q73" s="11" t="str">
         <x:v>releases/v7-3/assets/xiamen-detail-mask-7e7d2ac8b97d19f8.webp</x:v>
@@ -13149,7 +13200,7 @@
         <x:v>1217878</x:v>
       </x:c>
       <x:c r="P160" s="10" t="str">
-        <x:v>assets/xian-light-mask-c5024f591539dc71.webp</x:v>
+        <x:v>../v7-3/assets/xian-light-mask-c5024f591539dc71.webp</x:v>
       </x:c>
       <x:c r="Q160" s="10" t="str">
         <x:v>releases/v7-3/assets/xian-light-mask-c5024f591539dc71.webp</x:v>
@@ -13273,7 +13324,7 @@
         <x:v>4871510</x:v>
       </x:c>
       <x:c r="P162" s="10" t="str">
-        <x:v>assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
+        <x:v>../v7-3/assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
       </x:c>
       <x:c r="Q162" s="10" t="str">
         <x:v>releases/v7-3/assets/xian-standard-mask-6765eb28884cba73.webp</x:v>
@@ -13397,7 +13448,7 @@
         <x:v>19475115</x:v>
       </x:c>
       <x:c r="P164" s="10" t="str">
-        <x:v>assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
+        <x:v>../v7-3/assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
       </x:c>
       <x:c r="Q164" s="10" t="str">
         <x:v>releases/v7-3/assets/xian-detail-mask-2fec346956d39c3b.webp</x:v>
@@ -15257,7 +15308,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P194" s="10" t="str">
-        <x:v>assets/slogan-open-d0dc0df725a844be.webp</x:v>
+        <x:v>../v7-3/assets/slogan-open-d0dc0df725a844be.webp</x:v>
       </x:c>
       <x:c r="Q194" s="10" t="str">
         <x:v>releases/v7-3/assets/slogan-open-d0dc0df725a844be.webp</x:v>
@@ -15319,7 +15370,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P195" s="11" t="str">
-        <x:v>assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
+        <x:v>../v7-3/assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
       </x:c>
       <x:c r="Q195" s="11" t="str">
         <x:v>releases/v7-3/assets/slogan-innovation-0c31d18458db52dd.webp</x:v>
@@ -15381,7 +15432,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P196" s="10" t="str">
-        <x:v>assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
+        <x:v>../v7-3/assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
       </x:c>
       <x:c r="Q196" s="10" t="str">
         <x:v>releases/v7-3/assets/slogan-cooperation-e2c5f6b534591635.webp</x:v>
@@ -15443,7 +15494,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P197" s="11" t="str">
-        <x:v>assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
+        <x:v>../v7-3/assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
       </x:c>
       <x:c r="Q197" s="11" t="str">
         <x:v>releases/v7-3/assets/slogan-sharing-7d2d7bf570a46ce8.webp</x:v>
@@ -15505,7 +15556,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P198" s="10" t="str">
-        <x:v>assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
+        <x:v>../v7-3/assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
       </x:c>
       <x:c r="Q198" s="10" t="str">
         <x:v>releases/v7-3/assets/slogan-together-7e3a2c69d745a00f.webp</x:v>
@@ -15567,7 +15618,7 @@
         <x:v>359424</x:v>
       </x:c>
       <x:c r="P199" s="11" t="str">
-        <x:v>assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
+        <x:v>../v7-3/assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
       </x:c>
       <x:c r="Q199" s="11" t="str">
         <x:v>releases/v7-3/assets/slogan-ocean-4fcdcbb818dbd1a2.webp</x:v>
@@ -15647,7 +15698,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5978b9f9987444d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7a8dce8da364b54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
test(v7): verify final porcelain and high-detail feedback fixes
</commit_message>
<xml_diff>
--- a/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
+++ b/guangcai-china-preview/integration/backend-handoff/V7后台配置数据表.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="R7ca5b101c90c497d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="R1ed45773897b4d35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="R929891afc87b4b9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="R8e7899d0fdef472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="Rf0bd6d5736c54d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R8c557bba695d4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="录入说明与字段" sheetId="1" r:id="R8bf0f35535a34e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="城市配置" sheetId="2" r:id="Rc15ef6070e6b4215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颜色配置" sheetId="3" r:id="Rc6e3ab995c44455c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材质参数" sheetId="4" r:id="R42c33c4130c54043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="祝福语" sheetId="5" r:id="R35c75f47454040e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资源明细" sheetId="6" r:id="R35f2c5037a26410a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -609,7 +609,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1146,7 +1146,7 @@
         <x:v>CDN manifest</x:v>
       </x:c>
       <x:c r="H24" s="10" t="str">
-        <x:v>v7-4声明source-layout-v4：三部件花纹镜像，杯身花纹底边0.12 mm。缺省按v3。不是DesignConfig字段，不可由后台任意改写旧发布。</x:v>
+        <x:v>v7-4声明source-layout-v4：三部件花纹镜像，花纹底边0.12 mm，上连接白瓷下沿补足。缺省按v3。不是DesignConfig字段，不可由后台任意改写旧发布。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="55" customHeight="1">
@@ -1214,113 +1214,123 @@
         <x:v>数据来源（完整提交与文件哈希见JSON sources）</x:v>
       </x:c>
       <x:c r="H31" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/package.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/package.json</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
       <x:c r="H32" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.3/resource-build.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/evidence/v7.1.3/resource-build.json</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
       <x:c r="H33" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.3/handle-dimensions.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/evidence/v7.1.3/handle-dimensions.json</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
       <x:c r="H34" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/geometry/fixed-mapping.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/geometry/fixed-mapping.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
       <x:c r="H35" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/style-manager.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/geometry/product.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="34" customHeight="1">
       <x:c r="H36" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/integration/contracts/resource-manifest.schema.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/main.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="H37" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.2/slogans-source.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/styles/style-manager.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="H38" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/evidence/v7.1.2/cities/review.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/integration/contracts/resource-manifest.schema.json</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="H39" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/evidence/v7.1.2/slogans-source.json</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="H40" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/slogans.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/evidence/v7.1.2/cities/review.json</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
       <x:c r="H41" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/styles/city-appearance.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="H42" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/styles/slogans.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
       <x:c r="H43" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/styles/xy-mapping.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
       <x:c r="H44" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/ui/consumer-panel.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
       <x:c r="H45" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/types.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/styles/city-catalog-v6.json</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
       <x:c r="H46" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/design.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/materials/city-parametric.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
       <x:c r="H47" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/resources/types.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
       <x:c r="H48" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/resources/design.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="34" customHeight="1">
       <x:c r="H49" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/src/resources/texture-budget.ts</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="34" customHeight="1">
       <x:c r="H50" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/releases/v7-4/catalog.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/integration/contracts/design.schema.json</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="34" customHeight="1">
       <x:c r="H51" s="12" t="str">
-        <x:v>https://github.com/Shuang-su/guangcai/blob/3b7b509efe95034725ee655cc217badbc45f65bb/guangcai-china-preview/public/releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/public/api/v1/bootstrap.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="34" customHeight="1">
+      <x:c r="H52" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/public/releases/v7-4/catalog.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="34" customHeight="1">
+      <x:c r="H53" s="12" t="str">
+        <x:v>https://github.com/Shuang-su/guangcai/blob/d31e6821916c780ef7f8c1fc28add3252a8ff191/guangcai-china-preview/public/releases/v7-4/manifest-a6484ca5de3f4cc2.json</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reee7f11b36b347e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb1f3a65ce93475c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1378,7 +1388,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2395,7 +2405,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6a45a59bf5c4e10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8181358d08846bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2456,7 +2466,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2765,7 +2775,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdde0c29b00504b0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00eacb7d86cd4eaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2808,7 +2818,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3172,7 +3182,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c8aa1c35ee140dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re25b248403ad4e7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3215,7 +3225,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3420,7 +3430,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf7fc22a5fa146ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20189d526684991"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3499,7 +3509,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>V7.1.3 / v7-4 / 3b7b509efe95 · JSON为配置参考，作品接口保持原格式</x:v>
+        <x:v>V7.1.3 / v7-4 / d31e6821916c · JSON为配置参考，作品接口保持原格式</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -15698,7 +15708,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7a8dce8da364b54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92136639cd474216"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>